<commit_message>
feat(ai-sow): streamline owner handoffs and review flow
</commit_message>
<xml_diff>
--- a/plugins/ai-sow/skills/generate-sow/fixtures/project/.ai-sow/templates/sow-template.xlsx
+++ b/plugins/ai-sow/skills/generate-sow/fixtures/project/.ai-sow/templates/sow-template.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00-使用说明" sheetId="1" r:id="Ra0e2691636e84a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01-需求" sheetId="2" r:id="Re0d90c4a7eeb413e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02-子需求" sheetId="3" r:id="R6fbdd0a8e4a7402f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03-SOW主表" sheetId="4" r:id="Rdffbafb2ddda4454"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-验收条件" sheetId="5" r:id="Rac1e9d7c34554217"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05-任务明细" sheetId="6" r:id="R956f9a8429d24f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06-集成点" sheetId="7" r:id="R841601f7a1fe4b21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-假设清单" sheetId="8" r:id="R807d43a0ac8e4050"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20-项目汇总" sheetId="9" r:id="R131d303a23244b1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-系统现状" sheetId="10" r:id="R7dce5937ef1d4827"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="91-项目参数" sheetId="11" r:id="R8720a167bab04c80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="92-基础人天" sheetId="12" r:id="R62fba68f3f344516"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00-使用说明" sheetId="1" r:id="Raf46a5a6b82041f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01-需求" sheetId="2" r:id="R2d96ef47fa2e4a37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02-子需求" sheetId="3" r:id="R29f20c4962c446d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03-SOW主表" sheetId="4" r:id="R2ab7acc00eb54bb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-验收条件" sheetId="5" r:id="R601069b884ee4986"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05-任务明细" sheetId="6" r:id="Re439b5d6d8fe4771"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06-集成点" sheetId="7" r:id="Rfb4ed52343c742ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-假设清单" sheetId="8" r:id="R9e15ee74748c4f6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20-项目汇总" sheetId="9" r:id="R4bcda49c45c14c1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90-系统现状" sheetId="10" r:id="Rebd045ec577d4927"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="91-项目参数" sheetId="11" r:id="R2b0cf981975f4f67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="92-基础人天" sheetId="12" r:id="Rae55ac24257b4d9a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30,7 +30,7 @@
     <x:numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <x:numFmt numFmtId="200" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="52">
+  <x:fonts count="54">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -322,8 +322,19 @@
       <x:color rgb="FF667680"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF315F61"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF334155"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="107">
+  <x:fills count="110">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -855,6 +866,21 @@
         <x:fgColor rgb="FFFFF5E3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF26465F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F1F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="30">
     <x:border/>
@@ -1301,7 +1327,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="635">
+  <x:cellXfs count="647">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -2960,6 +2986,30 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="107" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="108" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="52" fillId="108" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="52" fillId="108" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="52" fillId="108" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="53" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="53" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="109" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
@@ -3013,7 +3063,7 @@
     <x:cellStyle name="40% - Accent6" xfId="47"/>
     <x:cellStyle name="60% - Accent6" xfId="48"/>
   </x:cellStyles>
-  <x:dxfs count="27">
+  <x:dxfs count="37">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -3290,6 +3340,106 @@
       </x:font>
       <x:fill>
         <x:patternFill>
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -4456,13 +4606,150 @@
     <x:row r="40" ht="68" customHeight="1"/>
     <x:row r="41" ht="68" customHeight="1"/>
     <x:row r="42" ht="68" customHeight="1"/>
-    <x:row r="43"/>
-    <x:row r="44" ht="42" customHeight="1"/>
-    <x:row r="45" ht="42" customHeight="1"/>
-    <x:row r="46" ht="42" customHeight="1"/>
-    <x:row r="47" ht="42" customHeight="1"/>
-    <x:row r="48" ht="42" customHeight="1"/>
-    <x:row r="49" ht="42" customHeight="1"/>
+    <x:row r="43">
+      <x:c r="A43" s="638" t="str">
+        <x:v>稳定输入 SHA-256</x:v>
+      </x:c>
+      <x:c r="B43" s="638"/>
+      <x:c r="C43" s="638"/>
+      <x:c r="D43" s="638"/>
+      <x:c r="E43" s="638"/>
+      <x:c r="F43" s="638"/>
+      <x:c r="G43" s="638"/>
+      <x:c r="H43" s="638"/>
+    </x:row>
+    <x:row r="44" ht="42" customHeight="1">
+      <x:c r="A44" s="642" t="str">
+        <x:v>sourceRequirements</x:v>
+      </x:c>
+      <x:c r="B44" s="646"/>
+      <x:c r="C44" s="646" t="str">
+        <x:v>Epic</x:v>
+      </x:c>
+      <x:c r="D44" s="646" t="str">
+        <x:v>无</x:v>
+      </x:c>
+      <x:c r="E44" s="646" t="str">
+        <x:v>稳定 ID</x:v>
+      </x:c>
+      <x:c r="F44" s="646" t="str">
+        <x:v>source/technical requirements</x:v>
+      </x:c>
+      <x:c r="G44" s="646" t="str">
+        <x:v>02-子需求</x:v>
+      </x:c>
+      <x:c r="H44" s="646"/>
+    </x:row>
+    <x:row r="45" ht="42" customHeight="1">
+      <x:c r="A45" s="642" t="str">
+        <x:v>asis</x:v>
+      </x:c>
+      <x:c r="B45" s="646"/>
+      <x:c r="C45" s="646" t="str">
+        <x:v>Epic</x:v>
+      </x:c>
+      <x:c r="D45" s="646" t="str">
+        <x:v>无</x:v>
+      </x:c>
+      <x:c r="E45" s="646" t="str">
+        <x:v>稳定 ID</x:v>
+      </x:c>
+      <x:c r="F45" s="646" t="str">
+        <x:v>source/technical requirements</x:v>
+      </x:c>
+      <x:c r="G45" s="646" t="str">
+        <x:v>02-子需求</x:v>
+      </x:c>
+      <x:c r="H45" s="646"/>
+    </x:row>
+    <x:row r="46" ht="42" customHeight="1">
+      <x:c r="A46" s="642" t="str">
+        <x:v>design</x:v>
+      </x:c>
+      <x:c r="B46" s="646"/>
+      <x:c r="C46" s="646" t="str">
+        <x:v>Epic</x:v>
+      </x:c>
+      <x:c r="D46" s="646" t="str">
+        <x:v>无</x:v>
+      </x:c>
+      <x:c r="E46" s="646" t="str">
+        <x:v>稳定 ID</x:v>
+      </x:c>
+      <x:c r="F46" s="646" t="str">
+        <x:v>source/technical requirements</x:v>
+      </x:c>
+      <x:c r="G46" s="646" t="str">
+        <x:v>02-子需求</x:v>
+      </x:c>
+      <x:c r="H46" s="646"/>
+    </x:row>
+    <x:row r="47" ht="42" customHeight="1">
+      <x:c r="A47" s="642" t="str">
+        <x:v>derivedRequirements</x:v>
+      </x:c>
+      <x:c r="B47" s="646"/>
+      <x:c r="C47" s="646" t="str">
+        <x:v>Epic</x:v>
+      </x:c>
+      <x:c r="D47" s="646" t="str">
+        <x:v>无</x:v>
+      </x:c>
+      <x:c r="E47" s="646" t="str">
+        <x:v>稳定 ID</x:v>
+      </x:c>
+      <x:c r="F47" s="646" t="str">
+        <x:v>source/technical requirements</x:v>
+      </x:c>
+      <x:c r="G47" s="646" t="str">
+        <x:v>02-子需求</x:v>
+      </x:c>
+      <x:c r="H47" s="646"/>
+    </x:row>
+    <x:row r="48" ht="42" customHeight="1">
+      <x:c r="A48" s="642" t="str">
+        <x:v>delivery</x:v>
+      </x:c>
+      <x:c r="B48" s="646"/>
+      <x:c r="C48" s="646" t="str">
+        <x:v>Epic</x:v>
+      </x:c>
+      <x:c r="D48" s="646" t="str">
+        <x:v>无</x:v>
+      </x:c>
+      <x:c r="E48" s="646" t="str">
+        <x:v>稳定 ID</x:v>
+      </x:c>
+      <x:c r="F48" s="646" t="str">
+        <x:v>source/technical requirements</x:v>
+      </x:c>
+      <x:c r="G48" s="646" t="str">
+        <x:v>02-子需求</x:v>
+      </x:c>
+      <x:c r="H48" s="646"/>
+    </x:row>
+    <x:row r="49" ht="42" customHeight="1">
+      <x:c r="A49" s="642" t="str">
+        <x:v>estimate</x:v>
+      </x:c>
+      <x:c r="B49" s="646"/>
+      <x:c r="C49" s="646" t="str">
+        <x:v>Epic</x:v>
+      </x:c>
+      <x:c r="D49" s="646" t="str">
+        <x:v>无</x:v>
+      </x:c>
+      <x:c r="E49" s="646" t="str">
+        <x:v>稳定 ID</x:v>
+      </x:c>
+      <x:c r="F49" s="646" t="str">
+        <x:v>source/technical requirements</x:v>
+      </x:c>
+      <x:c r="G49" s="646" t="str">
+        <x:v>02-子需求</x:v>
+      </x:c>
+      <x:c r="H49" s="646"/>
+    </x:row>
     <x:row r="50" ht="42" customHeight="1"/>
     <x:row r="51" ht="42" customHeight="1"/>
   </x:sheetData>
@@ -4804,8 +5091,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc29abec8dc0246d4"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf34d0b209359460e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9d54c43134a45cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8287957676db45e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5050,7 +5337,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R719cfe546fc946e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e33fdc8ab8e45a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9001,7 +9288,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fbca59d7bcb48a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99fd43458e37410e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9977,7 +10264,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R897d72f16902407e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd6e87a857ea4b7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11374,7 +11661,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a725de5514b4415"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b4af7ceae2a4be3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12837,9 +13124,9 @@
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="L5:L14">
-    <x:cfRule type="containsText" dxfId="19" priority="1" operator="containsText" text="已明确"/>
-    <x:cfRule type="containsText" dxfId="20" priority="2" operator="containsText" text="待确认"/>
+  <x:conditionalFormatting sqref="K5:K104">
+    <x:cfRule type="containsText" dxfId="35" priority="1" operator="containsText" text="已明确"/>
+    <x:cfRule type="containsText" dxfId="36" priority="2" operator="containsText" text="待确认"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C5:C104">
@@ -12851,7 +13138,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcbbad6a036145dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d4c4ff6ab81428f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13516,16 +13803,16 @@
     <x:mergeCell ref="A2:D2"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C5:C45">
-      <x:formula1>1</x:formula1>
-    </x:dataValidation>
     <x:dataValidation type="list" sqref="B5:B104">
       <x:formula1>INDIRECT("'03-SOW主表'!$A$5:$A$104")</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C5:C104">
+      <x:formula1>1</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e31d8311cf44cf9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f12c26d24ee4c36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22226,7 +22513,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b6b2ff3d3e84b17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcaa60815847a488b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23902,7 +24189,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e180945eb204e0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d019e6470fb4ff1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24008,7 +24295,7 @@
       <x:c r="G5" s="473" t="n"/>
       <x:c r="H5" s="461" t="n"/>
       <x:c r="I5" s="593" t="n">
-        <x:f>IF(OR(E5="",G5&lt;&gt;"待确认"),0,IFERROR(INDEX(SOWStoryTable[人天],MATCH(E5,SOWStoryTable[Story ID],0)),0))</x:f>
+        <x:f>IF(OR(E5="",G5&lt;&gt;"待确认"),0,SUMPRODUCT(SOWStoryTable[人天]*--ISNUMBER(SEARCH("、"&amp;SOWStoryTable[Story ID]&amp;"、","、"&amp;SUBSTITUTE(E5," ","")&amp;"、"))))</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -25123,7 +25410,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac488b788c844c19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9addb65d3bde4a26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25544,7 +25831,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21d4e14d17454298"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf91a9f46a1f04dca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>